<commit_message>
Actualizacion reglas lógicas V2
Se actualiza marcacion casa/comercio y se ajustan las reglas logicas con las variables de API
</commit_message>
<xml_diff>
--- a/data_simple_Team_72_EnergiAI/Matriz_Logica__Simple_EnergiAI_Teams_72.xlsx
+++ b/data_simple_Team_72_EnergiAI/Matriz_Logica__Simple_EnergiAI_Teams_72.xlsx
@@ -9,10 +9,11 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20400" windowHeight="7755" tabRatio="857"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20400" windowHeight="7755" tabRatio="857" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="matriz_logica_simple" sheetId="7" r:id="rId1"/>
+    <sheet name="matriz_logica_simpleV1" sheetId="8" r:id="rId1"/>
+    <sheet name="matriz_logica_simple V2" sheetId="7" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="67">
   <si>
     <t>Perfil Calculado</t>
   </si>
@@ -189,6 +190,42 @@
   </si>
   <si>
     <t>Ahorro est. $50.0 - $120.0 USD/mes (66.6 - 160.0 kwh/mes)</t>
+  </si>
+  <si>
+    <t>Casa</t>
+  </si>
+  <si>
+    <t>uso_horario_pico == True</t>
+  </si>
+  <si>
+    <t>(consumo_kwh / 30.0) &gt; 12.36 and horas_alto_consumo &gt; 6</t>
+  </si>
+  <si>
+    <t>(consumo_kwh / cantidad_equipos) &gt; 80.0</t>
+  </si>
+  <si>
+    <t>horas_alto_consumo &gt; 10</t>
+  </si>
+  <si>
+    <t>cantidad_equipos &gt;= 3 and (consumo_kwh / 30.0) &gt; 15.0</t>
+  </si>
+  <si>
+    <t>Comercio</t>
+  </si>
+  <si>
+    <t>uso_horario_pico == False and horas_alto_consumo &gt; 10</t>
+  </si>
+  <si>
+    <t>uso_horario_pico == True and horas_alto_consumo &gt; 8</t>
+  </si>
+  <si>
+    <t>horas_alto_consumo &gt; 12 and (consumo_kwh / cantidad_equipos) &gt; 60.0</t>
+  </si>
+  <si>
+    <t>superficie_m2 &gt; 0 and (consumo_kwh / superficie_m2) &gt; 22.76</t>
+  </si>
+  <si>
+    <t>Ineficiente</t>
   </si>
 </sst>
 </file>
@@ -795,4 +832,263 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46" customWidth="1"/>
+    <col min="3" max="3" width="38.42578125" customWidth="1"/>
+    <col min="4" max="4" width="39.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>